<commit_message>
feat: implement full-stack clinic management backend with patient and appointment services and a React simulation dashboard
</commit_message>
<xml_diff>
--- a/backend/data/clinic_data.xlsx
+++ b/backend/data/clinic_data.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -564,6 +564,92 @@
       <c r="M2" t="inlineStr">
         <is>
           <t>2026-09-05T20:56:49.996135</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PAT-000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dd</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>123456789</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>acknowledged</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:07:25.170585</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:07:25.170585</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PAT-000003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>naman</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1234567</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>acknowledged</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:11.292406</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:27.822949</t>
         </is>
       </c>
     </row>
@@ -764,7 +850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -776,13 +862,14 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -833,35 +920,40 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>booking_time</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>reason</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>review_notes</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>appointment_id</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
@@ -913,29 +1005,30 @@
           <t>13:00</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
         <is>
           <t>Dental Extraction</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>simulator</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr">
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
         <is>
           <t>2026-09-05T20:56:50.428206</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>2026-09-05T20:56:50.428206</t>
         </is>
@@ -987,29 +1080,30 @@
           <t>11:00</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
         <is>
           <t>Dental Consultation</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>simulator</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr">
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
         <is>
           <t>2026-09-05T20:57:35.307747</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>2026-09-05T20:57:35.307747</t>
         </is>
@@ -1061,31 +1155,498 @@
           <t>10:00</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
         <is>
           <t>Dental Consultation</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>simulator</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr">
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
         <is>
           <t>2026-09-05T20:58:08.219775</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>2026-09-05T20:58:08.219775</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>REQ-000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>dd</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>123456789</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PAT-000002</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>DOC-000002</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>General Checkup</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>simulator</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:07:25.685927</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:07:25.685927</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>REQ-000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>dd</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>123456789</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PAT-000002</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>DOC-000001</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Dental Consultation</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>simulator</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:07:46.846710</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:07:46.846710</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>REQ-000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>naman</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1234567</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PAT-000002</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>DOC-000002</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:11.761151</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>General Checkup</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>simulator</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:11.761151</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:11.761151</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>REQ-000007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>naman</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1234567</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>PAT-000002</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>DOC-000002</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:36.511224</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Dental Consultation</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>simulator</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:36.511224</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:36.511224</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>REQ-000008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>naman</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1234567</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PAT-000002</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>DOC-000001</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:49.931709</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Dental Consultation</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>simulator</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:49.931709</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:49.931709</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>REQ-000009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>naman</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1234567</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>PAT-000002</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>DOC-000002</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:40:30.142552</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Dental Consultation</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>simulator</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:40:30.142552</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:40:30.142552</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2017,16 +2578,17 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2062,50 +2624,55 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>booking_time</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>treatment_name</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>payment_status</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>bill_number</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>clinical_notes</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
@@ -2176,7 +2743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2370,6 +2937,302 @@
       <c r="G5" t="inlineStr">
         <is>
           <t>Patient request submitted from simulator for naman chauhan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LOG-000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:07:25.170585</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>staff_reception</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PATIENT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PAT-000002</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Registered patient dd (123456789)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LOG-000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:07:25.685927</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>simulator_bot</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PATIENT_REQUEST</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>REQ-000004</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Patient request submitted from simulator for dd</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LOG-000007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:07:46.846710</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>simulator_bot</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>PATIENT_REQUEST</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>REQ-000005</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Patient request submitted from simulator for dd</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LOG-000008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:11.292406</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>staff_reception</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PATIENT</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PAT-000003</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Registered patient naman (1234567)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LOG-000009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:11.761151</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>simulator_bot</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PATIENT_REQUEST</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>REQ-000006</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Patient request submitted from simulator for naman</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LOG-000010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:36.511224</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>simulator_bot</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>PATIENT_REQUEST</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>REQ-000007</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Patient request submitted from simulator for naman</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LOG-000011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:39:49.931709</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>simulator_bot</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PATIENT_REQUEST</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>REQ-000008</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Patient request submitted from simulator for naman</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LOG-000012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-05T21:40:30.142552</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>simulator_bot</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PATIENT_REQUEST</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>REQ-000009</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Patient request submitted from simulator for naman</t>
         </is>
       </c>
     </row>

</xml_diff>